<commit_message>
Make CAP box merging update live without re-render lag
</commit_message>
<xml_diff>
--- a/cap741-data.xlsx
+++ b/cap741-data.xlsx
@@ -10449,7 +10449,7 @@
         <v/>
       </c>
     </row>
-    <row r="243">
+    <row r="243" xml:space="preserve">
       <c r="A243" t="str">
         <v>Airbus A350-1000 - RR Trent XWB-97</v>
       </c>
@@ -10474,8 +10474,9 @@
       <c r="H243" t="str">
         <v>PERIODIC GROUND CHECK AT 7-DAY INTERVALS CARRIED OUT IAW DIR 10317077 PT 000 VERS 01. SEE SAP REVISION 01315524 DCN 001, 002 AND 003 FOR DETAILS</v>
       </c>
-      <c r="I243" t="str">
-        <v>Assisted with PERIODIC GROUND CHECK AT 7-DAY INTERVALS CARRIED OUT IAW DIR 10317077 PT 000 VERS 01. SEE SAP REVISION 01315524 DCN 001, 002 AND 003 FOR DETAILS for Action Maintenance Notification 40152456 - D7 NOTIFICATION, WBC STORAGE 7 DAY PE- D7 NOTIFICATION, W...c</v>
+      <c r="I243" t="str" xml:space="preserve">
+        <v xml:space="preserve">Assisted with PERIODIC GROUND CHECK AT 7-DAY INTERVALS CARRIED OUT IAW DIR 10317077 PT 000 VERS 01. SEE SAP REVISION 01315524 DCN 001, 002 AND 003 FOR DETAILS for Action Maintenance Notification 40152456 - D7 NOTIFICATION, WBC STORAGE 7 DAY PE- D7 NOTIFICATION, W...c
+Assisted with PERIODIC GROUND CHECK AT 7-DAY INTERVALS CARRIED OUT IAW DIR 10317077 PT 000 VERS 01. SEE SAP REVISION 01315524 DCN 001, 002 AND 003 FOR DETAILS for Action Maintenance Notification 40152456 - D7 NOTIFICATION, WBC STORAGE 7 DAY PE- D7 NOTIFICATION, W...c</v>
       </c>
       <c r="J243" t="str">
         <v>Kevin Cosgrave</v>
@@ -10487,7 +10488,7 @@
         <v>UK.66.412845A</v>
       </c>
       <c r="M243" t="str">
-        <v>true</v>
+        <v/>
       </c>
     </row>
     <row r="244">
@@ -15969,7 +15970,7 @@
         <v/>
       </c>
       <c r="I377" t="str">
-        <v>hello</v>
+        <v>hellovvv   tewrw</v>
       </c>
       <c r="J377" t="str">
         <v>David Needham</v>

</xml_diff>

<commit_message>
Add CAP741 Overlay preview
</commit_message>
<xml_diff>
--- a/cap741-data.xlsx
+++ b/cap741-data.xlsx
@@ -10449,7 +10449,7 @@
         <v/>
       </c>
     </row>
-    <row r="243" xml:space="preserve">
+    <row r="243">
       <c r="A243" t="str">
         <v>Airbus A350-1000 - RR Trent XWB-97</v>
       </c>
@@ -10474,9 +10474,8 @@
       <c r="H243" t="str">
         <v>PERIODIC GROUND CHECK AT 7-DAY INTERVALS CARRIED OUT IAW DIR 10317077 PT 000 VERS 01. SEE SAP REVISION 01315524 DCN 001, 002 AND 003 FOR DETAILS</v>
       </c>
-      <c r="I243" t="str" xml:space="preserve">
-        <v xml:space="preserve">Assisted with PERIODIC GROUND CHECK AT 7-DAY INTERVALS CARRIED OUT IAW DIR 10317077 PT 000 VERS 01. SEE SAP REVISION 01315524 DCN 001, 002 AND 003 FOR DETAILS for Action Maintenance Notification 40152456 - D7 NOTIFICATION, WBC STORAGE 7 DAY PE- D7 NOTIFICATION, W...c
-Assisted with PERIODIC GROUND CHECK AT 7-DAY INTERVALS CARRIED OUT IAW DIR 10317077 PT 000 VERS 01. SEE SAP REVISION 01315524 DCN 001, 002 AND 003 FOR DETAILS for Action Maintenance Notification 40152456 - D7 NOTIFICATION, WBC STORAGE 7 DAY PE- D7 NOTIFICATION, W...c</v>
+      <c r="I243" t="str">
+        <v>Assisted with PERIODIC GROUND CHECK AT 7-DAY INTERVALS CARRIED OUT IAW DIR 10317077 PT 000 VERS 01. SEE SAP REVISION 01315524 DCN 001, 002 AND 003 FOR DETAILS for Action Maintenance Notification 40152456 - D7 NOTIFICATION, WBC STORAGE 7 DAY PE- D7 NOTIFICATION, W...</v>
       </c>
       <c r="J243" t="str">
         <v>Kevin Cosgrave</v>

</xml_diff>

<commit_message>
keep the page fixed to A5
</commit_message>
<xml_diff>
--- a/cap741-data.xlsx
+++ b/cap741-data.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -470,7 +470,7 @@
         <v>Dummy data test one</v>
       </c>
       <c r="I2" t="str">
-        <v>Dummy data test one</v>
+        <v>Dummy data test one Dummy data test oneDummy data test oneDummy data test oneDummy data test oneDummy data test oneDummy data test oneDummy data test oneDummy data test oneDummy data test oneDummy data test oneDummy data test  test oneDummy data test oneDummy data test oneDummy data test one fgfgfgfgggg</v>
       </c>
       <c r="J2" t="str">
         <v>Ioannis Orkos</v>
@@ -485,9 +485,50 @@
         <v/>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v/>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v/>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix: preserve overlay print alignment by keeping table borders transparent
</commit_message>
<xml_diff>
--- a/cap741-data.xlsx
+++ b/cap741-data.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -446,10 +446,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v/>
+        <v>Airbus A350-1000 - RR Trent XWB-97</v>
       </c>
       <c r="B2" t="str">
-        <v/>
+        <v>G-XWBA</v>
       </c>
       <c r="C2" t="str">
         <v/>
@@ -485,57 +485,16 @@
         <v/>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v/>
-      </c>
-      <c r="B3" t="str">
-        <v/>
-      </c>
-      <c r="C3" t="str">
-        <v/>
-      </c>
-      <c r="D3" t="str">
-        <v/>
-      </c>
-      <c r="E3" t="str">
-        <v/>
-      </c>
-      <c r="F3" t="str">
-        <v/>
-      </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
-      <c r="H3" t="str">
-        <v/>
-      </c>
-      <c r="I3" t="str">
-        <v/>
-      </c>
-      <c r="J3" t="str">
-        <v/>
-      </c>
-      <c r="K3" t="str">
-        <v/>
-      </c>
-      <c r="L3" t="str">
-        <v/>
-      </c>
-      <c r="M3" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C88"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -548,16 +507,973 @@
         <v>Aircraft Type</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>A350</v>
+      </c>
+      <c r="B2" t="str">
+        <v>G-XWBA</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Airbus A350-1000 - RR Trent XWB-97</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>A350</v>
+      </c>
+      <c r="B3" t="str">
+        <v>G-XWBC</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Airbus A350-1000 - RR Trent XWB-97</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>A350</v>
+      </c>
+      <c r="B4" t="str">
+        <v>G-XWBD</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Airbus A350-1000 - RR Trent XWB-97</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>A350</v>
+      </c>
+      <c r="B5" t="str">
+        <v>G-XWBE</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Airbus A350-1000 - RR Trent XWB-97</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>A350</v>
+      </c>
+      <c r="B6" t="str">
+        <v>G-XWBF</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Airbus A350-1000 - RR Trent XWB-97</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>A350</v>
+      </c>
+      <c r="B7" t="str">
+        <v>G-XWBG</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Airbus A350-1000 - RR Trent XWB-97</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>A350</v>
+      </c>
+      <c r="B8" t="str">
+        <v>G-XWBK</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Airbus A350-1000 - RR Trent XWB-97</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>A350</v>
+      </c>
+      <c r="B9" t="str">
+        <v>G-XWBM</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Airbus A350-1000 - RR Trent XWB-97</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>A350</v>
+      </c>
+      <c r="B10" t="str">
+        <v>G-XWBS</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Airbus A350-1000 - RR Trent XWB-97</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>A380</v>
+      </c>
+      <c r="B11" t="str">
+        <v>G-XLEB</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Airbus A380-800 - RR Trent 900</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>A380</v>
+      </c>
+      <c r="B12" t="str">
+        <v>G-XLEC</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Airbus A380-800 - RR Trent 900</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>A380</v>
+      </c>
+      <c r="B13" t="str">
+        <v>G-XLED</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Airbus A380-800 - RR Trent 900</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>A380</v>
+      </c>
+      <c r="B14" t="str">
+        <v>G-XLEE</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Airbus A380-800 - RR Trent 900</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>A380</v>
+      </c>
+      <c r="B15" t="str">
+        <v>G-XLEF</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Airbus A380-800 - RR Trent 900</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>A380</v>
+      </c>
+      <c r="B16" t="str">
+        <v>G-XLEG</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Airbus A380-800 - RR Trent 900</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>A380</v>
+      </c>
+      <c r="B17" t="str">
+        <v>G-XLEH</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Airbus A380-800 - RR Trent 900</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>A380</v>
+      </c>
+      <c r="B18" t="str">
+        <v>G-XLEI</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Airbus A380-800 - RR Trent 900</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>A380</v>
+      </c>
+      <c r="B19" t="str">
+        <v>G-XLEJ</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Airbus A380-800 - RR Trent 900</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>A380</v>
+      </c>
+      <c r="B20" t="str">
+        <v>G-XLEK</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Airbus A380-800 - RR Trent 900</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>A380</v>
+      </c>
+      <c r="B21" t="str">
+        <v>G-XLEL</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Airbus A380-800 - RR Trent 900</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>B777 - GE90</v>
+      </c>
+      <c r="B22" t="str">
+        <v>G-STBC</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Boeing 777-300ER - GE90</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>B777 - GE90</v>
+      </c>
+      <c r="B23" t="str">
+        <v>G-STBE</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Boeing 777-300ER - GE90</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>B777 - GE90</v>
+      </c>
+      <c r="B24" t="str">
+        <v>G-STBF</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Boeing 777-300ER - GE90</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>B777 - GE90</v>
+      </c>
+      <c r="B25" t="str">
+        <v>G-STBG</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Boeing 777-300ER - GE90</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>B777 - GE90</v>
+      </c>
+      <c r="B26" t="str">
+        <v>G-STBH</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Boeing 777-300ER - GE90</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>B777 - GE90</v>
+      </c>
+      <c r="B27" t="str">
+        <v>G-STBK</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Boeing 777-300ER - GE90</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>B777 - GE90</v>
+      </c>
+      <c r="B28" t="str">
+        <v>G-STBL</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Boeing 777-300ER - GE90</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>B777 - GE90</v>
+      </c>
+      <c r="B29" t="str">
+        <v>G-STBM</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Boeing 777-300ER - GE90</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>B777 - GE90</v>
+      </c>
+      <c r="B30" t="str">
+        <v>G-STBN</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Boeing 777-300ER - GE90</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>B777 - GE90</v>
+      </c>
+      <c r="B31" t="str">
+        <v>G-STBO</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Boeing 777-300ER - GE90</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>B777 - GE90</v>
+      </c>
+      <c r="B32" t="str">
+        <v>G-VIIA</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Boeing 777-300ER - GE90</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>B777 - GE90</v>
+      </c>
+      <c r="B33" t="str">
+        <v>G-VIIB</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Boeing 777-300ER - GE90</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>B777 - GE90</v>
+      </c>
+      <c r="B34" t="str">
+        <v>G-VIIC</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Boeing 777-300ER - GE90</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>B777 - GE90</v>
+      </c>
+      <c r="B35" t="str">
+        <v>G-VIIE</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Boeing 777-300ER - GE90</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>B777 - GE90</v>
+      </c>
+      <c r="B36" t="str">
+        <v>G-VIIF</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Boeing 777-300ER - GE90</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>B777 - GE90</v>
+      </c>
+      <c r="B37" t="str">
+        <v>G-VIIG</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Boeing 777-300ER - GE90</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>B777 - GE90</v>
+      </c>
+      <c r="B38" t="str">
+        <v>G-VIIH</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Boeing 777-300ER - GE90</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>B777 - GE90</v>
+      </c>
+      <c r="B39" t="str">
+        <v>G-VIIJ</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Boeing 777-300ER - GE90</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>B777 - GE90</v>
+      </c>
+      <c r="B40" t="str">
+        <v>G-VIIK</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Boeing 777-300ER - GE90</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>B777 - GE90</v>
+      </c>
+      <c r="B41" t="str">
+        <v>G-VIIL</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Boeing 777-300ER - GE90</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>B777 - GE90</v>
+      </c>
+      <c r="B42" t="str">
+        <v>G-VIIN</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Boeing 777-300ER - GE90</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>B777 - GE90</v>
+      </c>
+      <c r="B43" t="str">
+        <v>G-VIIP</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Boeing 777-300ER - GE90</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>B777 - GE90</v>
+      </c>
+      <c r="B44" t="str">
+        <v>G-VIIS</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Boeing 777-300ER - GE90</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>B777 - GE90</v>
+      </c>
+      <c r="B45" t="str">
+        <v>G-VIIV</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Boeing 777-300ER - GE90</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>B777 - GE90</v>
+      </c>
+      <c r="B46" t="str">
+        <v>G-VIIW</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Boeing 777-300ER - GE90</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>B777 - Trent 800</v>
+      </c>
+      <c r="B47" t="str">
+        <v>G-YMMB</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Boeing 777-200ER - RR Trent 800</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>B777 - Trent 800</v>
+      </c>
+      <c r="B48" t="str">
+        <v>G-YMMF</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Boeing 777-200ER - RR Trent 800</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>B777 - Trent 800</v>
+      </c>
+      <c r="B49" t="str">
+        <v>G-YMMG</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Boeing 777-200ER - RR Trent 800</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>B777 - Trent 800</v>
+      </c>
+      <c r="B50" t="str">
+        <v>G-YMMI</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Boeing 777-200ER - RR Trent 800</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>B777 - Trent 800</v>
+      </c>
+      <c r="B51" t="str">
+        <v>G-YMMJ</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Boeing 777-200ER - RR Trent 800</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>B777 - Trent 800</v>
+      </c>
+      <c r="B52" t="str">
+        <v>G-YMMK</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Boeing 777-200ER - RR Trent 800</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>B777 - Trent 800</v>
+      </c>
+      <c r="B53" t="str">
+        <v>G-YMMP</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Boeing 777-200ER - RR Trent 800</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>B777 - Trent 800</v>
+      </c>
+      <c r="B54" t="str">
+        <v>G-YMMT</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Boeing 777-200ER - RR Trent 800</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>B777 - Trent 800</v>
+      </c>
+      <c r="B55" t="str">
+        <v>G-YMMU</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Boeing 777-200ER - RR Trent 800</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B56" t="str">
+        <v>G-ZBJA</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Boeing 787-8 - RR Trent 1000</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B57" t="str">
+        <v>G-ZBJB</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Boeing 787-8 - RR Trent 1000</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B58" t="str">
+        <v>G-ZBJC</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Boeing 787-8 - RR Trent 1000</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B59" t="str">
+        <v>G-ZBJD</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Boeing 787-8 - RR Trent 1000</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B60" t="str">
+        <v>G-ZBJE</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Boeing 787-8 - RR Trent 1000</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B61" t="str">
+        <v>G-ZBJG</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Boeing 787-8 - RR Trent 1000</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B62" t="str">
+        <v>G-ZBJH</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Boeing 787-8 - RR Trent 1000</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B63" t="str">
+        <v>G-ZBJI</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Boeing 787-8 - RR Trent 1000</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B64" t="str">
+        <v>G-ZBJJ</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Boeing 787-8 - RR Trent 1000</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B65" t="str">
+        <v>G-ZBJK</v>
+      </c>
+      <c r="C65" t="str">
+        <v>Boeing 787-8 - RR Trent 1000</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B66" t="str">
+        <v>G-ZBKA</v>
+      </c>
+      <c r="C66" t="str">
+        <v>Boeing 787-9 - RR Trent 1000</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B67" t="str">
+        <v>G-ZBKB</v>
+      </c>
+      <c r="C67" t="str">
+        <v>Boeing 787-9 - RR Trent 1000</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B68" t="str">
+        <v>G-ZBKC</v>
+      </c>
+      <c r="C68" t="str">
+        <v>Boeing 787-9 - RR Trent 1000</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B69" t="str">
+        <v>G-ZBKD</v>
+      </c>
+      <c r="C69" t="str">
+        <v>Boeing 787-9 - RR Trent 1000</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B70" t="str">
+        <v>G-ZBKE</v>
+      </c>
+      <c r="C70" t="str">
+        <v>Boeing 787-9 - RR Trent 1000</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B71" t="str">
+        <v>G-ZBKF</v>
+      </c>
+      <c r="C71" t="str">
+        <v>Boeing 787-9 - RR Trent 1000</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B72" t="str">
+        <v>G-ZBKH</v>
+      </c>
+      <c r="C72" t="str">
+        <v>Boeing 787-9 - RR Trent 1000</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B73" t="str">
+        <v>G-ZBKI</v>
+      </c>
+      <c r="C73" t="str">
+        <v>Boeing 787-9 - RR Trent 1000</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B74" t="str">
+        <v>G-ZBKJ</v>
+      </c>
+      <c r="C74" t="str">
+        <v>Boeing 787-9 - RR Trent 1000</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B75" t="str">
+        <v>G-ZBKK</v>
+      </c>
+      <c r="C75" t="str">
+        <v>Boeing 787-9 - RR Trent 1000</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B76" t="str">
+        <v>G-ZBKL</v>
+      </c>
+      <c r="C76" t="str">
+        <v>Boeing 787-9 - RR Trent 1000</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B77" t="str">
+        <v>G-ZBKM</v>
+      </c>
+      <c r="C77" t="str">
+        <v>Boeing 787-9 - RR Trent 1000</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B78" t="str">
+        <v>G-ZBKN</v>
+      </c>
+      <c r="C78" t="str">
+        <v>Boeing 787-9 - RR Trent 1000</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B79" t="str">
+        <v>G-ZBKO</v>
+      </c>
+      <c r="C79" t="str">
+        <v>Boeing 787-9 - RR Trent 1000</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B80" t="str">
+        <v>G-ZBKR</v>
+      </c>
+      <c r="C80" t="str">
+        <v>Boeing 787-9 - RR Trent 1000</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B81" t="str">
+        <v>G-ZBKS</v>
+      </c>
+      <c r="C81" t="str">
+        <v>Boeing 787-9 - RR Trent 1000</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B82" t="str">
+        <v>G-ZBLA</v>
+      </c>
+      <c r="C82" t="str">
+        <v>Boeing 787-10 - RR Trent 1000</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B83" t="str">
+        <v>G-ZBLB</v>
+      </c>
+      <c r="C83" t="str">
+        <v>Boeing 787-10 - RR Trent 1000</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B84" t="str">
+        <v>G-ZBLC</v>
+      </c>
+      <c r="C84" t="str">
+        <v>Boeing 787-10 - RR Trent 1000</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B85" t="str">
+        <v>G-ZBLE</v>
+      </c>
+      <c r="C85" t="str">
+        <v>Boeing 787-10 - RR Trent 1000</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B86" t="str">
+        <v>G-ZBLF</v>
+      </c>
+      <c r="C86" t="str">
+        <v>Boeing 787-10 - RR Trent 1000</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B87" t="str">
+        <v>G-ZBLG</v>
+      </c>
+      <c r="C87" t="str">
+        <v>Boeing 787-10 - RR Trent 1000</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>B787</v>
+      </c>
+      <c r="B88" t="str">
+        <v>G-ZBLH</v>
+      </c>
+      <c r="C88" t="str">
+        <v>Boeing 787-10 - RR Trent 1000</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C88"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B82"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -567,9 +1483,657 @@
         <v>Description</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>00</v>
+      </c>
+      <c r="B2" t="str">
+        <v>General</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>01</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Maintenance Policy</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>02</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Operations</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>03</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Support</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>04</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Airworthiness Limitations</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>05</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Time Limits / Maintenance Checks</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>06</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Dimensions and Areas</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>07</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Lifting and Shoring</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>08</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Leveling and Weighing</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>09</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Towing and Taxiing</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>10</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Parking, Mooring, Storage and Return To Service</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>11</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Placards and Markings</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>12</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Servicing</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>13</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Hardware and General Tools</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Aircrew Information</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>16</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Change of Role</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>18</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Vibration and Noise Analysis</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>20</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Standard Practices - Airframe</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>21</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Air Conditioning and Pressurization</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>22</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Auto Flight</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>23</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Communications</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>24</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Electrical Power</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>25</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Equipment / Furnishings</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>26</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Fire Protection</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>27</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Flight Controls</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>28</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Fuel</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>29</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Hydraulic Power</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>30</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Ice and Rain Protection</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>31</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Indicating / Recording Systems</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>32</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Landing Gear</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>33</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Lights</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>34</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Navigation</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>35</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Oxygen</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>36</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Pneumatic</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>37</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Vacuum</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>38</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Water / Waste</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>39</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Electrical - Electronic Panels and Multipurpose Components</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>40</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Multisystem</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>41</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Water Ballast</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>42</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Integrated Modular Avionics (IMA)</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>43</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Emergency Solar Panel System (ESPS)</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>44</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Cabin Systems</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>45</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Central Maintenance / Onboard Maintenance Systems</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>46</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Information Systems</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>47</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Nitrogen Generation / Inert Gas System</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>48</v>
+      </c>
+      <c r="B47" t="str">
+        <v>In Flight Fuel Dispensing</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>49</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Airborne Auxiliary Power</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>50</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Cargo and Accessory Compartments</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>51</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Standard Practices and Structures - General</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>52</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Doors</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>53</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Fuselage</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>54</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Nacelles / Pylons</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>55</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Stabilizers</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>56</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Windows</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>57</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Wings</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>60</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Standard Practices - Prop./Rotor</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>61</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Propellers / Propulsion</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>62</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Main Rotor(s)</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>63</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Main Rotor Drive(s)</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>64</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Tail Rotor</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>65</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Tail Rotor Drive</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>66</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Folding Blades / Pylon</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>67</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Rotors Flight Control</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>70</v>
+      </c>
+      <c r="B65" t="str">
+        <v>Standard Practices - Engine</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>71</v>
+      </c>
+      <c r="B66" t="str">
+        <v>Power Plant</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>72</v>
+      </c>
+      <c r="B67" t="str">
+        <v>Engine</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>73</v>
+      </c>
+      <c r="B68" t="str">
+        <v>Engine - Fuel and Control</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>74</v>
+      </c>
+      <c r="B69" t="str">
+        <v>Ignition</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>75</v>
+      </c>
+      <c r="B70" t="str">
+        <v>Bleed Air</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>76</v>
+      </c>
+      <c r="B71" t="str">
+        <v>Engine Controls</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>77</v>
+      </c>
+      <c r="B72" t="str">
+        <v>Engine Indicating</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>78</v>
+      </c>
+      <c r="B73" t="str">
+        <v>Exhaust</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>79</v>
+      </c>
+      <c r="B74" t="str">
+        <v>Oil</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>80</v>
+      </c>
+      <c r="B75" t="str">
+        <v>Starting</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>81</v>
+      </c>
+      <c r="B76" t="str">
+        <v>Turbines (Reciprocating Engines)</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>82</v>
+      </c>
+      <c r="B77" t="str">
+        <v>Water Injection</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>83</v>
+      </c>
+      <c r="B78" t="str">
+        <v>Accessory Gear Box (Engine Driven)</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>84</v>
+      </c>
+      <c r="B79" t="str">
+        <v>Propulsion Augmentation</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>85</v>
+      </c>
+      <c r="B80" t="str">
+        <v>Reciprocating Engine</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>91</v>
+      </c>
+      <c r="B81" t="str">
+        <v>Charts</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>97</v>
+      </c>
+      <c r="B82" t="str">
+        <v>Image Recording</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B82"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: add workbook-backed flags with modal picker, settings tab, and page badges
</commit_message>
<xml_diff>
--- a/cap741-data.xlsx
+++ b/cap741-data.xlsx
@@ -7,7 +7,8 @@
     <sheet name="Aircraft" sheetId="2" r:id="rId2"/>
     <sheet name="Chapters" sheetId="3" r:id="rId3"/>
     <sheet name="Supervisors" sheetId="4" r:id="rId4"/>
-    <sheet name="Info" sheetId="5" r:id="rId5"/>
+    <sheet name="Flags" sheetId="5" r:id="rId5"/>
+    <sheet name="Info" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -401,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:N2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -432,15 +433,18 @@
         <v>Rewriten for cap741</v>
       </c>
       <c r="J1" t="str">
+        <v>Flags</v>
+      </c>
+      <c r="K1" t="str">
         <v>Approval Name</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>Approval stamp</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>Aprroval Licence No.</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>Signed</v>
       </c>
     </row>
@@ -473,21 +477,24 @@
         <v>Dummy data test one Dummy data test oneDummy data test oneDummy data test oneDummy data test oneDummy data test oneDummy data test oneDummy data test oneDummy data test oneDummy data test oneDummy data test oneDummy data test  test oneDummy data test oneDummy data test oneDummy data test one fgfgfgfgggg</v>
       </c>
       <c r="J2" t="str">
-        <v>Ioannis Orkos</v>
+        <v>INSP - Inspections (Surveillance, Detailed &amp; General Visual); T/S - Troubleshooting</v>
       </c>
       <c r="K2" t="str">
         <v>Ioannis Orkos</v>
       </c>
       <c r="L2" t="str">
+        <v>Ioannis Orkos</v>
+      </c>
+      <c r="M2" t="str">
         <v>UK.XX.XXXXXXX</v>
       </c>
-      <c r="M2" t="str">
+      <c r="N2" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2191,7 +2198,172 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:C14"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Section</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Flag</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Color</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Primary</v>
+      </c>
+      <c r="B2" t="str">
+        <v>INSP - Inspections (Surveillance, Detailed &amp; General Visual)</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Gold</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Primary</v>
+      </c>
+      <c r="B3" t="str">
+        <v>T/S - Troubleshooting</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Purple</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Primary</v>
+      </c>
+      <c r="B4" t="str">
+        <v>F &amp; O - Functional &amp; Operational Check</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Green</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Primary</v>
+      </c>
+      <c r="B5" t="str">
+        <v>SRM - Structural Repair Manual</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Blue</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Primary</v>
+      </c>
+      <c r="B6" t="str">
+        <v>R &amp; I - Removal &amp; Installation</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Maroon</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>More</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Metal Damage Assessment*</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Black</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>More</v>
+      </c>
+      <c r="B8" t="str">
+        <v>CDCCL Tasks*</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Gray</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>More</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Metal Repair*</v>
+      </c>
+      <c r="C9" t="str">
+        <v>MistyRose</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>More</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Elect Wiring, Looming, Crimping, Soldering etc.*</v>
+      </c>
+      <c r="C10" t="str">
+        <v>SkyBlue</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>More</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Composite Damage Assessment*</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Teal</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>More</v>
+      </c>
+      <c r="B12" t="str">
+        <v>ESDS Procedures*</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Pink</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>More</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Composite Repair*</v>
+      </c>
+      <c r="C13" t="str">
+        <v>DarkRed</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>More</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Avionic LRU Replacement*</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Aqua</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C14"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2225,9 +2397,25 @@
         <v>User User</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Show Mind Map</v>
+      </c>
+      <c r="B5" t="str">
+        <v>true</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Page Grouping</v>
+      </c>
+      <c r="B6" t="str">
+        <v>type</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>